<commit_message>
Miễn thuế đến 15.4
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F3662E-187B-40AA-96CA-759E11C97F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431A524F-16E6-42C1-A525-52C96846DFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1900,9 +1900,6 @@
       <c r="A10" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="B10" s="6">
-        <v>1000</v>
-      </c>
       <c r="D10" s="4" t="s">
         <v>40</v>
       </c>
@@ -1937,9 +1934,6 @@
       <c r="A11" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="B11" s="6">
-        <v>1900</v>
-      </c>
       <c r="D11" s="5" t="s">
         <v>44</v>
       </c>
@@ -1973,9 +1967,6 @@
       <c r="A12" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="B12" s="6">
-        <v>2000</v>
-      </c>
       <c r="D12" s="5" t="s">
         <v>48</v>
       </c>
@@ -2008,9 +1999,6 @@
     <row r="13" spans="1:16" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>222</v>
-      </c>
-      <c r="B13" s="6">
-        <v>1000</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Dọn dẹp - Thuế MT 0
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431A524F-16E6-42C1-A525-52C96846DFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93366DB7-241F-4147-8B51-7B00052ADBDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="371">
   <si>
     <t>Mã kho</t>
   </si>
@@ -1138,6 +1138,18 @@
   </si>
   <si>
     <t>HH050-039</t>
+  </si>
+  <si>
+    <t>Quất Lâm</t>
+  </si>
+  <si>
+    <t>KDNL081</t>
+  </si>
+  <si>
+    <t>1K26TQL</t>
+  </si>
+  <si>
+    <t>KKKNT</t>
   </si>
 </sst>
 </file>
@@ -1900,6 +1912,9 @@
       <c r="A10" s="6" t="s">
         <v>223</v>
       </c>
+      <c r="B10" s="6">
+        <v>0</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>40</v>
       </c>
@@ -1934,6 +1949,9 @@
       <c r="A11" s="6" t="s">
         <v>224</v>
       </c>
+      <c r="B11" s="6">
+        <v>0</v>
+      </c>
       <c r="D11" s="5" t="s">
         <v>44</v>
       </c>
@@ -1967,6 +1985,9 @@
       <c r="A12" s="6" t="s">
         <v>225</v>
       </c>
+      <c r="B12" s="6">
+        <v>0</v>
+      </c>
       <c r="D12" s="5" t="s">
         <v>48</v>
       </c>
@@ -1999,6 +2020,9 @@
     <row r="13" spans="1:16" s="6" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>222</v>
+      </c>
+      <c r="B13" s="6">
+        <v>0</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>53</v>
@@ -2288,8 +2312,8 @@
       <c r="A22" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="1">
-        <v>8</v>
+      <c r="B22" s="1" t="s">
+        <v>370</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>98</v>
@@ -3146,6 +3170,21 @@
         <v>131114</v>
       </c>
       <c r="C46" s="10"/>
+      <c r="D46" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="47" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">

</xml_diff>

<commit_message>
Bổ sung Hợp Hưng Trường Thi
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D90DE3F-F230-4120-B389-B5D3B07BD0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A555939-9953-4751-A783-F63116A950F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="445">
   <si>
     <t>Mã kho</t>
   </si>
@@ -1300,6 +1300,78 @@
   </si>
   <si>
     <t>HH0642</t>
+  </si>
+  <si>
+    <t>Thiên Tôn</t>
+  </si>
+  <si>
+    <t>KDNL184</t>
+  </si>
+  <si>
+    <t>KDNL084</t>
+  </si>
+  <si>
+    <t>1K26TAG</t>
+  </si>
+  <si>
+    <t>HH009-009</t>
+  </si>
+  <si>
+    <t>HH050-044</t>
+  </si>
+  <si>
+    <t>HH051-047</t>
+  </si>
+  <si>
+    <t>KDNL181</t>
+  </si>
+  <si>
+    <t>Hợp Hưng</t>
+  </si>
+  <si>
+    <t>Trường Thi</t>
+  </si>
+  <si>
+    <t>KDNL185</t>
+  </si>
+  <si>
+    <t>KDNL186</t>
+  </si>
+  <si>
+    <t>KDNL085</t>
+  </si>
+  <si>
+    <t>KDNL086</t>
+  </si>
+  <si>
+    <t>1K26THH</t>
+  </si>
+  <si>
+    <t>1K26THI</t>
+  </si>
+  <si>
+    <t>HH009-010</t>
+  </si>
+  <si>
+    <t>HH050-045</t>
+  </si>
+  <si>
+    <t>HH051-048</t>
+  </si>
+  <si>
+    <t>HH0645</t>
+  </si>
+  <si>
+    <t>HH009-011</t>
+  </si>
+  <si>
+    <t>HH050-046</t>
+  </si>
+  <si>
+    <t>HH051-050</t>
+  </si>
+  <si>
+    <t>HH0646</t>
   </si>
 </sst>
 </file>
@@ -3467,7 +3539,7 @@
         <v>374</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>368</v>
+        <v>428</v>
       </c>
       <c r="L46" s="1" t="s">
         <v>369</v>
@@ -3484,6 +3556,30 @@
         <v>221</v>
       </c>
       <c r="B47" s="10"/>
+      <c r="D47" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="48" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10" t="s">
@@ -3492,16 +3588,70 @@
       <c r="B48" s="10">
         <v>3338111</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D48" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="M48" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N48" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10" t="s">
         <v>34</v>
       </c>
       <c r="B49" s="10">
         <v>3338121</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="M49" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10" t="s">
         <v>11</v>
       </c>
@@ -3509,7 +3659,7 @@
         <v>333814</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>220</v>
       </c>
@@ -3517,13 +3667,13 @@
         <v>63211</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>168</v>
       </c>
       <c r="B52" s="10"/>
     </row>
-    <row r="53" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10" t="s">
         <v>18</v>
       </c>
@@ -3531,7 +3681,7 @@
         <v>333111</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10" t="s">
         <v>34</v>
       </c>
@@ -3539,7 +3689,7 @@
         <v>333112</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Fix MVV Mỹ Xá
</commit_message>
<xml_diff>
--- a/Data_HDDT.xlsx
+++ b/Data_HDDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A555939-9953-4751-A783-F63116A950F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C87EF8-F5E1-4E92-8AC9-78784AF4E205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1224,9 +1224,6 @@
     <t>HH051-008</t>
   </si>
   <si>
-    <t>HH051-001</t>
-  </si>
-  <si>
     <t>HH051-017</t>
   </si>
   <si>
@@ -1372,6 +1369,9 @@
   </si>
   <si>
     <t>HH0646</t>
+  </si>
+  <si>
+    <t>HH051-010</t>
   </si>
 </sst>
 </file>
@@ -2659,7 +2659,7 @@
         <v>106</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>395</v>
+        <v>444</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>190</v>
@@ -2694,7 +2694,7 @@
         <v>280</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>199</v>
@@ -2729,7 +2729,7 @@
         <v>275</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>198</v>
@@ -2768,7 +2768,7 @@
         <v>232</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>213</v>
@@ -2803,7 +2803,7 @@
         <v>125</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>211</v>
@@ -2839,7 +2839,7 @@
         <v>130</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>212</v>
@@ -2880,7 +2880,7 @@
         <v>135</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>214</v>
@@ -2921,7 +2921,7 @@
         <v>347</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>204</v>
@@ -2962,7 +2962,7 @@
         <v>144</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>186</v>
@@ -3001,7 +3001,7 @@
         <v>150</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>215</v>
@@ -3039,7 +3039,7 @@
         <v>154</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>206</v>
@@ -3077,7 +3077,7 @@
         <v>158</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>216</v>
@@ -3115,7 +3115,7 @@
         <v>162</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>195</v>
@@ -3153,7 +3153,7 @@
         <v>167</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>203</v>
@@ -3192,7 +3192,7 @@
         <v>278</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>184</v>
@@ -3233,7 +3233,7 @@
         <v>284</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>218</v>
@@ -3274,7 +3274,7 @@
         <v>281</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>201</v>
@@ -3313,7 +3313,7 @@
         <v>290</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="J40" s="1" t="s">
         <v>291</v>
@@ -3347,7 +3347,7 @@
         <v>297</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>298</v>
@@ -3383,7 +3383,7 @@
         <v>304</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>305</v>
@@ -3419,7 +3419,7 @@
         <v>349</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>352</v>
@@ -3457,10 +3457,10 @@
         <v>356</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="K44" s="1" t="s">
         <v>357</v>
@@ -3495,10 +3495,10 @@
         <v>366</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>361</v>
@@ -3533,13 +3533,13 @@
         <v>373</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J46" s="1" t="s">
         <v>374</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="L46" s="1" t="s">
         <v>369</v>
@@ -3557,28 +3557,28 @@
       </c>
       <c r="B47" s="10"/>
       <c r="D47" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="K47" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G47" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="I47" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N47" s="1" t="s">
         <v>422</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="M47" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="N47" s="1" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
@@ -3589,31 +3589,31 @@
         <v>3338111</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G48" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="H48" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="H48" s="1" t="s">
+      <c r="I48" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="I48" s="1" t="s">
+      <c r="J48" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="J48" s="1" t="s">
-        <v>440</v>
-      </c>
       <c r="K48" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="M48" s="1" t="s">
         <v>18</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
@@ -3624,31 +3624,31 @@
         <v>3338121</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="G49" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="H49" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="I49" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="I49" s="1" t="s">
+      <c r="J49" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="J49" s="1" t="s">
-        <v>444</v>
-      </c>
       <c r="K49" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="M49" s="1" t="s">
         <v>18</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>